<commit_message>
Update to 6 query sheets in Excel output
</commit_message>
<xml_diff>
--- a/s&p_500_analysis.xlsx
+++ b/s&p_500_analysis.xlsx
@@ -10,6 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buy Dips" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avg Price per Sector" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top Market Cap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non volatile" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="One year change" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top Sellers" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +441,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>AVG(Price)</t>
+          <t>Price</t>
         </is>
       </c>
     </row>
@@ -861,4 +864,354 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>AVG(PE_Ratio)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>18.04903846153846</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-37.871</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>39.90382352941177</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>24.84575757575758</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>40.64217391304349</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>30.49368421052631</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>59.1525</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>52.64666666666667</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>17.08769230769231</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>322.24</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>-179.93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>AVG(Change_1Y)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.051014285714287</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.3941818181818181</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.3192151898734176</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.3096153846153845</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.2083125</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.1645483870967742</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.15252</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.08447457627118644</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.02867741935483871</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>-0.02847222222222222</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Volume_1D</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>201.68</v>
+      </c>
+      <c r="C2" t="n">
+        <v>147784255</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>97.31</v>
+      </c>
+      <c r="C3" t="n">
+        <v>115213495</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>111196199</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>